<commit_message>
docs: VFO+keyer order — add Digi-Key P/N column alongside Mouser
VFO_Keyer_Order.xlsx and tools/gen_vfo_keyer_order.py: added a
Digi-Key P/N column next to the existing Mouser P/N column so the
sheet can be used to fill either supplier's cart depending on stock
availability. Renamed "Supplier" to "Ordered From" — fill in after
the PO to track which vendor actually shipped.

Populated Digi-Key P/Ns where reliably known (active devices, IC
sockets, headers, silver mica caps, X7R / tantalum bypass, BNC,
zener, film cap, paddle/standoff hardware). Left blank for Yageo
MFR-25 axial resistors (DK catalog number varies per value — easier
to search by spec) and KitsAndParts-only items (toroids, magnet
wire). Updated Instructions sheet to explain the gaps.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/VFO_Keyer_Order.xlsx
+++ b/Documentation/VFO_Keyer_Order.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -542,11 +542,12 @@
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -592,25 +593,30 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Ordered From</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Part Number</t>
+          <t>Mouser P/N</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Digi-Key P/N</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Unit $</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Ext $</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -638,6 +644,7 @@
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -666,26 +673,23 @@
       <c r="F3" s="7" t="inlineStr"/>
       <c r="G3" s="7" t="inlineStr"/>
       <c r="H3" s="7" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>Adafruit</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>5566</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n">
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>1528-5566-ND</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="n">
         <v>11.95</v>
       </c>
-      <c r="L3" s="8">
-        <f>E3*K3</f>
-        <v/>
-      </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>OWN this already; verify P/N</t>
+      <c r="M3" s="8">
+        <f>E3*L3</f>
+        <v/>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>OWN this; Adafruit P/N 5566. Adafruit-only part.</t>
         </is>
       </c>
     </row>
@@ -716,24 +720,25 @@
       <c r="F4" s="7" t="inlineStr"/>
       <c r="G4" s="7" t="inlineStr"/>
       <c r="H4" s="7" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr">
         <is>
           <t>855-R30-1001003</t>
         </is>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>36-3475-ND</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="n">
         <v>0.6</v>
       </c>
-      <c r="L4" s="8">
-        <f>E4*K4</f>
-        <v/>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="8">
+        <f>E4*L4</f>
+        <v/>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Corner standoffs for Si5351</t>
         </is>
@@ -766,24 +771,25 @@
       <c r="F5" s="7" t="inlineStr"/>
       <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr">
         <is>
           <t>534-29390</t>
         </is>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>36-29390-ND</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="L5" s="8">
-        <f>E5*K5</f>
-        <v/>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M5" s="8">
+        <f>E5*L5</f>
+        <v/>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>2 per standoff</t>
         </is>
@@ -816,24 +822,21 @@
       <c r="F6" s="7" t="inlineStr"/>
       <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr">
         <is>
           <t>602-9314-4-100-NC025</t>
         </is>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="L6" s="8">
-        <f>E6*K6</f>
-        <v/>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M6" s="8">
+        <f>E6*L6</f>
+        <v/>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>For 7 jumpers Si5351 to PCB + general use</t>
         </is>
@@ -861,6 +864,7 @@
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -889,24 +893,21 @@
       <c r="F8" s="7" t="inlineStr"/>
       <c r="G8" s="7" t="inlineStr"/>
       <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FBF52-0R0</t>
         </is>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L8" s="8">
-        <f>E8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="8">
+        <f>E8*L8</f>
+        <v/>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>Optional damper, default 0R</t>
         </is>
@@ -939,24 +940,21 @@
       <c r="F9" s="7" t="inlineStr"/>
       <c r="G9" s="7" t="inlineStr"/>
       <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
           <t>581-SR152A103JAR</t>
         </is>
       </c>
-      <c r="K9" s="8" t="n">
+      <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="8" t="n">
         <v>0.45</v>
       </c>
-      <c r="L9" s="8">
-        <f>E9*K9</f>
-        <v/>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="8">
+        <f>E9*L9</f>
+        <v/>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>Si5351 CLK0 to pi pad coupling; blocks 1.65V offset</t>
         </is>
@@ -989,24 +987,21 @@
       <c r="F10" s="7" t="inlineStr"/>
       <c r="G10" s="7" t="inlineStr"/>
       <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-62R</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L10" s="8">
-        <f>E10*K10</f>
-        <v/>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="8">
+        <f>E10*L10</f>
+        <v/>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>Pi pad input shunt</t>
         </is>
@@ -1039,24 +1034,21 @@
       <c r="F11" s="7" t="inlineStr"/>
       <c r="G11" s="7" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-240R</t>
         </is>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L11" s="8">
-        <f>E11*K11</f>
-        <v/>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="8">
+        <f>E11*L11</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>Pi pad series</t>
         </is>
@@ -1089,24 +1081,21 @@
       <c r="F12" s="7" t="inlineStr"/>
       <c r="G12" s="7" t="inlineStr"/>
       <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-62R</t>
         </is>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L12" s="8">
-        <f>E12*K12</f>
-        <v/>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="8">
+        <f>E12*L12</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>Pi pad output shunt</t>
         </is>
@@ -1139,24 +1128,25 @@
       <c r="F13" s="7" t="inlineStr"/>
       <c r="G13" s="7" t="inlineStr"/>
       <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr">
         <is>
           <t>598-CD15FD221JO3F</t>
         </is>
       </c>
-      <c r="K13" s="8" t="n">
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>CD15FD221JO3F-ND</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="n">
         <v>1.85</v>
       </c>
-      <c r="L13" s="8">
-        <f>E13*K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="8">
+        <f>E13*L13</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>LPF outer; surplus item 189 (240pF) acceptable</t>
         </is>
@@ -1189,24 +1179,25 @@
       <c r="F14" s="7" t="inlineStr"/>
       <c r="G14" s="7" t="inlineStr"/>
       <c r="H14" s="7" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr">
         <is>
           <t>598-CD15FD391JO3F</t>
         </is>
       </c>
-      <c r="K14" s="8" t="n">
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>CD15FD391JO3F-ND</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="n">
         <v>1.95</v>
       </c>
-      <c r="L14" s="8">
-        <f>E14*K14</f>
-        <v/>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="8">
+        <f>E14*L14</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>LPF; surplus item 192 exact match</t>
         </is>
@@ -1239,24 +1230,25 @@
       <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="5" t="inlineStr">
         <is>
           <t>598-CD15FD391JO3F</t>
         </is>
       </c>
-      <c r="K15" s="8" t="n">
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>CD15FD391JO3F-ND</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="n">
         <v>1.95</v>
       </c>
-      <c r="L15" s="8">
-        <f>E15*K15</f>
-        <v/>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="8">
+        <f>E15*L15</f>
+        <v/>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>LPF; surplus item 192 exact match</t>
         </is>
@@ -1289,24 +1281,25 @@
       <c r="F16" s="7" t="inlineStr"/>
       <c r="G16" s="7" t="inlineStr"/>
       <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr">
         <is>
           <t>598-CD15FD221JO3F</t>
         </is>
       </c>
-      <c r="K16" s="8" t="n">
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>CD15FD221JO3F-ND</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="n">
         <v>1.85</v>
       </c>
-      <c r="L16" s="8">
-        <f>E16*K16</f>
-        <v/>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="8">
+        <f>E16*L16</f>
+        <v/>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>Same as CF1</t>
         </is>
@@ -1339,26 +1332,19 @@
       <c r="F17" s="7" t="inlineStr"/>
       <c r="G17" s="7" t="inlineStr"/>
       <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>KitsAndParts</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>T68-6</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="n">
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="8" t="n">
         <v>0.85</v>
       </c>
-      <c r="L17" s="8">
-        <f>E17*K17</f>
-        <v/>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
-        <is>
-          <t>3 inductors + 2 spares for redos</t>
+      <c r="M17" s="8">
+        <f>E17*L17</f>
+        <v/>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>KitsAndParts.com only - neither Mouser nor DK stocks Micrometals cores</t>
         </is>
       </c>
     </row>
@@ -1389,26 +1375,19 @@
       <c r="F18" s="7" t="inlineStr"/>
       <c r="G18" s="7" t="inlineStr"/>
       <c r="H18" s="7" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr">
-        <is>
-          <t>KitsAndParts</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>#24 1/4lb</t>
-        </is>
-      </c>
-      <c r="K18" s="8" t="n">
+      <c r="I18" s="7" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L18" s="8">
-        <f>E18*K18</f>
-        <v/>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
-        <is>
-          <t>Covers all 3 VFO LPF toroid windings</t>
+      <c r="M18" s="8">
+        <f>E18*L18</f>
+        <v/>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>KitsAndParts.com - neither Mouser nor DK stocks ham magnet wire</t>
         </is>
       </c>
     </row>
@@ -1439,26 +1418,23 @@
       <c r="F19" s="7" t="inlineStr"/>
       <c r="G19" s="7" t="inlineStr"/>
       <c r="H19" s="7" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-49R9</t>
         </is>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L19" s="8">
-        <f>E19*K19</f>
-        <v/>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
-        <is>
-          <t>LPF output termination</t>
+      <c r="M19" s="8">
+        <f>E19*L19</f>
+        <v/>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>LPF output termination (49.9 ohm = nearest E96)</t>
         </is>
       </c>
     </row>
@@ -1489,24 +1465,21 @@
       <c r="F20" s="7" t="inlineStr"/>
       <c r="G20" s="7" t="inlineStr"/>
       <c r="H20" s="7" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I20" s="7" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-1M</t>
         </is>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L20" s="8">
-        <f>E20*K20</f>
-        <v/>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M20" s="8">
+        <f>E20*L20</f>
+        <v/>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>MC1496 carrier-port grid-leak; ADD TO SCH</t>
         </is>
@@ -1534,6 +1507,7 @@
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1562,24 +1536,25 @@
       <c r="F22" s="7" t="inlineStr"/>
       <c r="G22" s="7" t="inlineStr"/>
       <c r="H22" s="7" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I22" s="7" t="inlineStr"/>
       <c r="J22" s="5" t="inlineStr">
         <is>
           <t>512-J310</t>
         </is>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>J310-ND</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="n">
         <v>0.85</v>
       </c>
-      <c r="L22" s="8">
-        <f>E22*K22</f>
-        <v/>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M22" s="8">
+        <f>E22*L22</f>
+        <v/>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>1 + 1 spare; static-sensitive</t>
         </is>
@@ -1612,24 +1587,21 @@
       <c r="F23" s="7" t="inlineStr"/>
       <c r="G23" s="7" t="inlineStr"/>
       <c r="H23" s="7" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="5" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-270R</t>
         </is>
       </c>
-      <c r="K23" s="8" t="n">
+      <c r="K23" s="5" t="inlineStr"/>
+      <c r="L23" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="L23" s="8">
-        <f>E23*K23</f>
-        <v/>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="M23" s="8">
+        <f>E23*L23</f>
+        <v/>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>J310 source resistor</t>
         </is>
@@ -1662,24 +1634,21 @@
       <c r="F24" s="7" t="inlineStr"/>
       <c r="G24" s="7" t="inlineStr"/>
       <c r="H24" s="7" t="inlineStr"/>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I24" s="7" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr">
         <is>
           <t>581-SR152A103JAR</t>
         </is>
       </c>
-      <c r="K24" s="8" t="n">
+      <c r="K24" s="5" t="inlineStr"/>
+      <c r="L24" s="8" t="n">
         <v>0.45</v>
       </c>
-      <c r="L24" s="8">
-        <f>E24*K24</f>
-        <v/>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="M24" s="8">
+        <f>E24*L24</f>
+        <v/>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>J310 output coupling to MC1496</t>
         </is>
@@ -1707,6 +1676,7 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -1735,24 +1705,25 @@
       <c r="F26" s="7" t="inlineStr"/>
       <c r="G26" s="7" t="inlineStr"/>
       <c r="H26" s="7" t="inlineStr"/>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I26" s="7" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr">
         <is>
           <t>511-MC1496P</t>
         </is>
       </c>
-      <c r="K26" s="11" t="n">
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>MC1496PG-ND</t>
+        </is>
+      </c>
+      <c r="L26" s="11" t="n">
         <v>2.45</v>
       </c>
-      <c r="L26" s="11">
-        <f>E26*K26</f>
-        <v/>
-      </c>
-      <c r="M26" s="9" t="inlineStr">
+      <c r="M26" s="11">
+        <f>E26*L26</f>
+        <v/>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
         <is>
           <t>1 + 1 spare; static-sensitive</t>
         </is>
@@ -1785,26 +1756,27 @@
       <c r="F27" s="7" t="inlineStr"/>
       <c r="G27" s="7" t="inlineStr"/>
       <c r="H27" s="7" t="inlineStr"/>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I27" s="7" t="inlineStr"/>
       <c r="J27" s="9" t="inlineStr">
         <is>
           <t>575-1102873</t>
         </is>
       </c>
-      <c r="K27" s="11" t="n">
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>AE9990-ND</t>
+        </is>
+      </c>
+      <c r="L27" s="11" t="n">
         <v>0.85</v>
       </c>
-      <c r="L27" s="11">
-        <f>E27*K27</f>
-        <v/>
-      </c>
-      <c r="M27" s="9" t="inlineStr">
-        <is>
-          <t>Mill-Max preferred</t>
+      <c r="M27" s="11">
+        <f>E27*L27</f>
+        <v/>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>Mill-Max machined preferred over stamped</t>
         </is>
       </c>
     </row>
@@ -1835,24 +1807,21 @@
       <c r="F28" s="7" t="inlineStr"/>
       <c r="G28" s="7" t="inlineStr"/>
       <c r="H28" s="7" t="inlineStr"/>
-      <c r="I28" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I28" s="7" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-51R</t>
         </is>
       </c>
-      <c r="K28" s="11" t="n">
+      <c r="K28" s="9" t="inlineStr"/>
+      <c r="L28" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L28" s="11">
-        <f>E28*K28</f>
-        <v/>
-      </c>
-      <c r="M28" s="9" t="inlineStr">
+      <c r="M28" s="11">
+        <f>E28*L28</f>
+        <v/>
+      </c>
+      <c r="N28" s="9" t="inlineStr">
         <is>
           <t>MC1496 carrier port termination</t>
         </is>
@@ -1885,24 +1854,21 @@
       <c r="F29" s="7" t="inlineStr"/>
       <c r="G29" s="7" t="inlineStr"/>
       <c r="H29" s="7" t="inlineStr"/>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I29" s="7" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-6K8</t>
         </is>
       </c>
-      <c r="K29" s="11" t="n">
+      <c r="K29" s="9" t="inlineStr"/>
+      <c r="L29" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L29" s="11">
-        <f>E29*K29</f>
-        <v/>
-      </c>
-      <c r="M29" s="9" t="inlineStr">
+      <c r="M29" s="11">
+        <f>E29*L29</f>
+        <v/>
+      </c>
+      <c r="N29" s="9" t="inlineStr">
         <is>
           <t>MC1496 Iee setting (pin 5)</t>
         </is>
@@ -1935,24 +1901,21 @@
       <c r="F30" s="7" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr"/>
       <c r="H30" s="7" t="inlineStr"/>
-      <c r="I30" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I30" s="7" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-51R</t>
         </is>
       </c>
-      <c r="K30" s="11" t="n">
+      <c r="K30" s="9" t="inlineStr"/>
+      <c r="L30" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L30" s="11">
-        <f>E30*K30</f>
-        <v/>
-      </c>
-      <c r="M30" s="9" t="inlineStr">
+      <c r="M30" s="11">
+        <f>E30*L30</f>
+        <v/>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
         <is>
           <t>MC1496 modulator port</t>
         </is>
@@ -1985,24 +1948,21 @@
       <c r="F31" s="7" t="inlineStr"/>
       <c r="G31" s="7" t="inlineStr"/>
       <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I31" s="7" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-51R</t>
         </is>
       </c>
-      <c r="K31" s="11" t="n">
+      <c r="K31" s="9" t="inlineStr"/>
+      <c r="L31" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L31" s="11">
-        <f>E31*K31</f>
-        <v/>
-      </c>
-      <c r="M31" s="9" t="inlineStr">
+      <c r="M31" s="11">
+        <f>E31*L31</f>
+        <v/>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
         <is>
           <t>Modulator port + DAC injection shunt at pin 1</t>
         </is>
@@ -2035,24 +1995,21 @@
       <c r="F32" s="7" t="inlineStr"/>
       <c r="G32" s="7" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr"/>
-      <c r="I32" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I32" s="7" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-3K9</t>
         </is>
       </c>
-      <c r="K32" s="11" t="n">
+      <c r="K32" s="9" t="inlineStr"/>
+      <c r="L32" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L32" s="11">
-        <f>E32*K32</f>
-        <v/>
-      </c>
-      <c r="M32" s="9" t="inlineStr">
+      <c r="M32" s="11">
+        <f>E32*L32</f>
+        <v/>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
         <is>
           <t>Output load; order 4-5 and match by DMM</t>
         </is>
@@ -2085,24 +2042,21 @@
       <c r="F33" s="7" t="inlineStr"/>
       <c r="G33" s="7" t="inlineStr"/>
       <c r="H33" s="7" t="inlineStr"/>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-3K9</t>
         </is>
       </c>
-      <c r="K33" s="11" t="n">
+      <c r="K33" s="9" t="inlineStr"/>
+      <c r="L33" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L33" s="11">
-        <f>E33*K33</f>
-        <v/>
-      </c>
-      <c r="M33" s="9" t="inlineStr">
+      <c r="M33" s="11">
+        <f>E33*L33</f>
+        <v/>
+      </c>
+      <c r="N33" s="9" t="inlineStr">
         <is>
           <t>See RLa note</t>
         </is>
@@ -2135,24 +2089,21 @@
       <c r="F34" s="7" t="inlineStr"/>
       <c r="G34" s="7" t="inlineStr"/>
       <c r="H34" s="7" t="inlineStr"/>
-      <c r="I34" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I34" s="7" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-8K2</t>
         </is>
       </c>
-      <c r="K34" s="11" t="n">
+      <c r="K34" s="9" t="inlineStr"/>
+      <c r="L34" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L34" s="11">
-        <f>E34*K34</f>
-        <v/>
-      </c>
-      <c r="M34" s="9" t="inlineStr">
+      <c r="M34" s="11">
+        <f>E34*L34</f>
+        <v/>
+      </c>
+      <c r="N34" s="9" t="inlineStr">
         <is>
           <t>PNP T1 base (symmetry)</t>
         </is>
@@ -2185,24 +2136,21 @@
       <c r="F35" s="7" t="inlineStr"/>
       <c r="G35" s="7" t="inlineStr"/>
       <c r="H35" s="7" t="inlineStr"/>
-      <c r="I35" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I35" s="7" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-8K2</t>
         </is>
       </c>
-      <c r="K35" s="11" t="n">
+      <c r="K35" s="9" t="inlineStr"/>
+      <c r="L35" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L35" s="11">
-        <f>E35*K35</f>
-        <v/>
-      </c>
-      <c r="M35" s="9" t="inlineStr">
+      <c r="M35" s="11">
+        <f>E35*L35</f>
+        <v/>
+      </c>
+      <c r="N35" s="9" t="inlineStr">
         <is>
           <t>PNP T2 base (symmetry; match R5)</t>
         </is>
@@ -2235,24 +2183,21 @@
       <c r="F36" s="7" t="inlineStr"/>
       <c r="G36" s="7" t="inlineStr"/>
       <c r="H36" s="7" t="inlineStr"/>
-      <c r="I36" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-8K2</t>
         </is>
       </c>
-      <c r="K36" s="11" t="n">
+      <c r="K36" s="9" t="inlineStr"/>
+      <c r="L36" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L36" s="11">
-        <f>E36*K36</f>
-        <v/>
-      </c>
-      <c r="M36" s="9" t="inlineStr">
+      <c r="M36" s="11">
+        <f>E36*L36</f>
+        <v/>
+      </c>
+      <c r="N36" s="9" t="inlineStr">
         <is>
           <t>PNP null injection</t>
         </is>
@@ -2285,24 +2230,21 @@
       <c r="F37" s="7" t="inlineStr"/>
       <c r="G37" s="7" t="inlineStr"/>
       <c r="H37" s="7" t="inlineStr"/>
-      <c r="I37" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I37" s="7" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-8K2</t>
         </is>
       </c>
-      <c r="K37" s="11" t="n">
+      <c r="K37" s="9" t="inlineStr"/>
+      <c r="L37" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L37" s="11">
-        <f>E37*K37</f>
-        <v/>
-      </c>
-      <c r="M37" s="9" t="inlineStr">
+      <c r="M37" s="11">
+        <f>E37*L37</f>
+        <v/>
+      </c>
+      <c r="N37" s="9" t="inlineStr">
         <is>
           <t>PNP null injection</t>
         </is>
@@ -2335,24 +2277,21 @@
       <c r="F38" s="7" t="inlineStr"/>
       <c r="G38" s="7" t="inlineStr"/>
       <c r="H38" s="7" t="inlineStr"/>
-      <c r="I38" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I38" s="7" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-2K7</t>
         </is>
       </c>
-      <c r="K38" s="11" t="n">
+      <c r="K38" s="9" t="inlineStr"/>
+      <c r="L38" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L38" s="11">
-        <f>E38*K38</f>
-        <v/>
-      </c>
-      <c r="M38" s="9" t="inlineStr">
+      <c r="M38" s="11">
+        <f>E38*L38</f>
+        <v/>
+      </c>
+      <c r="N38" s="9" t="inlineStr">
         <is>
           <t>PNP T1 collector bias</t>
         </is>
@@ -2385,24 +2324,21 @@
       <c r="F39" s="7" t="inlineStr"/>
       <c r="G39" s="7" t="inlineStr"/>
       <c r="H39" s="7" t="inlineStr"/>
-      <c r="I39" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-2K7</t>
         </is>
       </c>
-      <c r="K39" s="11" t="n">
+      <c r="K39" s="9" t="inlineStr"/>
+      <c r="L39" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L39" s="11">
-        <f>E39*K39</f>
-        <v/>
-      </c>
-      <c r="M39" s="9" t="inlineStr">
+      <c r="M39" s="11">
+        <f>E39*L39</f>
+        <v/>
+      </c>
+      <c r="N39" s="9" t="inlineStr">
         <is>
           <t>PNP T2 collector bias (match R6_K)</t>
         </is>
@@ -2435,24 +2371,21 @@
       <c r="F40" s="7" t="inlineStr"/>
       <c r="G40" s="7" t="inlineStr"/>
       <c r="H40" s="7" t="inlineStr"/>
-      <c r="I40" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I40" s="7" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-22K</t>
         </is>
       </c>
-      <c r="K40" s="11" t="n">
+      <c r="K40" s="9" t="inlineStr"/>
+      <c r="L40" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L40" s="11">
-        <f>E40*K40</f>
-        <v/>
-      </c>
-      <c r="M40" s="9" t="inlineStr">
+      <c r="M40" s="11">
+        <f>E40*L40</f>
+        <v/>
+      </c>
+      <c r="N40" s="9" t="inlineStr">
         <is>
           <t>Carrier bias divider top</t>
         </is>
@@ -2485,24 +2418,21 @@
       <c r="F41" s="7" t="inlineStr"/>
       <c r="G41" s="7" t="inlineStr"/>
       <c r="H41" s="7" t="inlineStr"/>
-      <c r="I41" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I41" s="7" t="inlineStr"/>
       <c r="J41" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-22K</t>
         </is>
       </c>
-      <c r="K41" s="11" t="n">
+      <c r="K41" s="9" t="inlineStr"/>
+      <c r="L41" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L41" s="11">
-        <f>E41*K41</f>
-        <v/>
-      </c>
-      <c r="M41" s="9" t="inlineStr">
+      <c r="M41" s="11">
+        <f>E41*L41</f>
+        <v/>
+      </c>
+      <c r="N41" s="9" t="inlineStr">
         <is>
           <t>Carrier bias divider bottom</t>
         </is>
@@ -2535,24 +2465,21 @@
       <c r="F42" s="7" t="inlineStr"/>
       <c r="G42" s="7" t="inlineStr"/>
       <c r="H42" s="7" t="inlineStr"/>
-      <c r="I42" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I42" s="7" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-1K5</t>
         </is>
       </c>
-      <c r="K42" s="11" t="n">
+      <c r="K42" s="9" t="inlineStr"/>
+      <c r="L42" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L42" s="11">
-        <f>E42*K42</f>
-        <v/>
-      </c>
-      <c r="M42" s="9" t="inlineStr">
+      <c r="M42" s="11">
+        <f>E42*L42</f>
+        <v/>
+      </c>
+      <c r="N42" s="9" t="inlineStr">
         <is>
           <t>Modulator input divider</t>
         </is>
@@ -2585,24 +2512,21 @@
       <c r="F43" s="7" t="inlineStr"/>
       <c r="G43" s="7" t="inlineStr"/>
       <c r="H43" s="7" t="inlineStr"/>
-      <c r="I43" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I43" s="7" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-2K</t>
         </is>
       </c>
-      <c r="K43" s="11" t="n">
+      <c r="K43" s="9" t="inlineStr"/>
+      <c r="L43" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L43" s="11">
-        <f>E43*K43</f>
-        <v/>
-      </c>
-      <c r="M43" s="9" t="inlineStr">
+      <c r="M43" s="11">
+        <f>E43*L43</f>
+        <v/>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
         <is>
           <t>MC1496 emitter degen (gain set)</t>
         </is>
@@ -2635,24 +2559,21 @@
       <c r="F44" s="7" t="inlineStr"/>
       <c r="G44" s="7" t="inlineStr"/>
       <c r="H44" s="7" t="inlineStr"/>
-      <c r="I44" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I44" s="7" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr">
         <is>
           <t>581-SR152A331JAR</t>
         </is>
       </c>
-      <c r="K44" s="11" t="n">
+      <c r="K44" s="9" t="inlineStr"/>
+      <c r="L44" s="11" t="n">
         <v>0.45</v>
       </c>
-      <c r="L44" s="11">
-        <f>E44*K44</f>
-        <v/>
-      </c>
-      <c r="M44" s="9" t="inlineStr">
+      <c r="M44" s="11">
+        <f>E44*L44</f>
+        <v/>
+      </c>
+      <c r="N44" s="9" t="inlineStr">
         <is>
           <t>Carrier port coupling; surplus item 191 also fine</t>
         </is>
@@ -2685,24 +2606,25 @@
       <c r="F45" s="7" t="inlineStr"/>
       <c r="G45" s="7" t="inlineStr"/>
       <c r="H45" s="7" t="inlineStr"/>
-      <c r="I45" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I45" s="7" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr">
         <is>
           <t>80-C320C104K5R</t>
         </is>
       </c>
-      <c r="K45" s="11" t="n">
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>399-9866-ND</t>
+        </is>
+      </c>
+      <c r="L45" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="L45" s="11">
-        <f>E45*K45</f>
-        <v/>
-      </c>
-      <c r="M45" s="9" t="inlineStr">
+      <c r="M45" s="11">
+        <f>E45*L45</f>
+        <v/>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
         <is>
           <t>MC1496 pin 10 bypass + 1 spare</t>
         </is>
@@ -2735,24 +2657,25 @@
       <c r="F46" s="7" t="inlineStr"/>
       <c r="G46" s="7" t="inlineStr"/>
       <c r="H46" s="7" t="inlineStr"/>
-      <c r="I46" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I46" s="7" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr">
         <is>
           <t>610-2N3906</t>
         </is>
       </c>
-      <c r="K46" s="11" t="n">
+      <c r="K46" s="9" t="inlineStr">
+        <is>
+          <t>2N3906FS-ND</t>
+        </is>
+      </c>
+      <c r="L46" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="L46" s="11">
-        <f>E46*K46</f>
-        <v/>
-      </c>
-      <c r="M46" s="9" t="inlineStr">
+      <c r="M46" s="11">
+        <f>E46*L46</f>
+        <v/>
+      </c>
+      <c r="N46" s="9" t="inlineStr">
         <is>
           <t>PNP null injection; buy 4 and pair by Vbe</t>
         </is>
@@ -2785,11 +2708,12 @@
       <c r="F47" s="7" t="inlineStr"/>
       <c r="G47" s="7" t="inlineStr"/>
       <c r="H47" s="7" t="inlineStr"/>
-      <c r="I47" s="9" t="inlineStr"/>
+      <c r="I47" s="7" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
-      <c r="K47" s="10" t="n"/>
+      <c r="K47" s="9" t="inlineStr"/>
       <c r="L47" s="10" t="n"/>
-      <c r="M47" s="9" t="inlineStr">
+      <c r="M47" s="10" t="n"/>
+      <c r="N47" s="9" t="inlineStr">
         <is>
           <t>Paired with T1 from the 4 ordered</t>
         </is>
@@ -2817,6 +2741,7 @@
       <c r="K48" s="3" t="n"/>
       <c r="L48" s="3" t="n"/>
       <c r="M48" s="3" t="n"/>
+      <c r="N48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
@@ -2845,24 +2770,25 @@
       <c r="F49" s="7" t="inlineStr"/>
       <c r="G49" s="7" t="inlineStr"/>
       <c r="H49" s="7" t="inlineStr"/>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I49" s="7" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr">
         <is>
           <t>926-LM7171AIN/NOPB</t>
         </is>
       </c>
-      <c r="K49" s="11" t="n">
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>LM7171AIN/NOPB-ND</t>
+        </is>
+      </c>
+      <c r="L49" s="11" t="n">
         <v>7.95</v>
       </c>
-      <c r="L49" s="11">
-        <f>E49*K49</f>
-        <v/>
-      </c>
-      <c r="M49" s="9" t="inlineStr">
+      <c r="M49" s="11">
+        <f>E49*L49</f>
+        <v/>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
         <is>
           <t>2 needed + 1 spare</t>
         </is>
@@ -2895,24 +2821,25 @@
       <c r="F50" s="7" t="inlineStr"/>
       <c r="G50" s="7" t="inlineStr"/>
       <c r="H50" s="7" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I50" s="7" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr">
         <is>
           <t>575-1102871</t>
         </is>
       </c>
-      <c r="K50" s="11" t="n">
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>AE9986-ND</t>
+        </is>
+      </c>
+      <c r="L50" s="11" t="n">
         <v>0.55</v>
       </c>
-      <c r="L50" s="11">
-        <f>E50*K50</f>
-        <v/>
-      </c>
-      <c r="M50" s="9" t="inlineStr">
+      <c r="M50" s="11">
+        <f>E50*L50</f>
+        <v/>
+      </c>
+      <c r="N50" s="9" t="inlineStr">
         <is>
           <t>For LM7171 x 2 + MCP4921</t>
         </is>
@@ -2945,24 +2872,25 @@
       <c r="F51" s="7" t="inlineStr"/>
       <c r="G51" s="7" t="inlineStr"/>
       <c r="H51" s="7" t="inlineStr"/>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I51" s="7" t="inlineStr"/>
       <c r="J51" s="9" t="inlineStr">
         <is>
           <t>80-C320C104K5R</t>
         </is>
       </c>
-      <c r="K51" s="11" t="n">
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>399-9866-ND</t>
+        </is>
+      </c>
+      <c r="L51" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="L51" s="11">
-        <f>E51*K51</f>
-        <v/>
-      </c>
-      <c r="M51" s="9" t="inlineStr">
+      <c r="M51" s="11">
+        <f>E51*L51</f>
+        <v/>
+      </c>
+      <c r="N51" s="9" t="inlineStr">
         <is>
           <t>2 per LM7171 input AC couple</t>
         </is>
@@ -2995,24 +2923,25 @@
       <c r="F52" s="7" t="inlineStr"/>
       <c r="G52" s="7" t="inlineStr"/>
       <c r="H52" s="7" t="inlineStr"/>
-      <c r="I52" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I52" s="7" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr">
         <is>
           <t>80-C320C104K5R</t>
         </is>
       </c>
-      <c r="K52" s="11" t="n">
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>399-9866-ND</t>
+        </is>
+      </c>
+      <c r="L52" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="L52" s="11">
-        <f>E52*K52</f>
-        <v/>
-      </c>
-      <c r="M52" s="9" t="inlineStr">
+      <c r="M52" s="11">
+        <f>E52*L52</f>
+        <v/>
+      </c>
+      <c r="N52" s="9" t="inlineStr">
         <is>
           <t>2 per LM7171 output AC couple</t>
         </is>
@@ -3045,24 +2974,21 @@
       <c r="F53" s="7" t="inlineStr"/>
       <c r="G53" s="7" t="inlineStr"/>
       <c r="H53" s="7" t="inlineStr"/>
-      <c r="I53" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I53" s="7" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-100K</t>
         </is>
       </c>
-      <c r="K53" s="11" t="n">
+      <c r="K53" s="9" t="inlineStr"/>
+      <c r="L53" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L53" s="11">
-        <f>E53*K53</f>
-        <v/>
-      </c>
-      <c r="M53" s="9" t="inlineStr">
+      <c r="M53" s="11">
+        <f>E53*L53</f>
+        <v/>
+      </c>
+      <c r="N53" s="9" t="inlineStr">
         <is>
           <t>LM7171 input bias</t>
         </is>
@@ -3095,24 +3021,21 @@
       <c r="F54" s="7" t="inlineStr"/>
       <c r="G54" s="7" t="inlineStr"/>
       <c r="H54" s="7" t="inlineStr"/>
-      <c r="I54" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I54" s="7" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-47K</t>
         </is>
       </c>
-      <c r="K54" s="11" t="n">
+      <c r="K54" s="9" t="inlineStr"/>
+      <c r="L54" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L54" s="11">
-        <f>E54*K54</f>
-        <v/>
-      </c>
-      <c r="M54" s="9" t="inlineStr">
+      <c r="M54" s="11">
+        <f>E54*L54</f>
+        <v/>
+      </c>
+      <c r="N54" s="9" t="inlineStr">
         <is>
           <t>LM7171 feedback (gain 5.8)</t>
         </is>
@@ -3145,24 +3068,21 @@
       <c r="F55" s="7" t="inlineStr"/>
       <c r="G55" s="7" t="inlineStr"/>
       <c r="H55" s="7" t="inlineStr"/>
-      <c r="I55" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I55" s="7" t="inlineStr"/>
       <c r="J55" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-10K</t>
         </is>
       </c>
-      <c r="K55" s="11" t="n">
+      <c r="K55" s="9" t="inlineStr"/>
+      <c r="L55" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L55" s="11">
-        <f>E55*K55</f>
-        <v/>
-      </c>
-      <c r="M55" s="9" t="inlineStr">
+      <c r="M55" s="11">
+        <f>E55*L55</f>
+        <v/>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
         <is>
           <t>LM7171 inverting leg to GND</t>
         </is>
@@ -3190,6 +3110,7 @@
       <c r="K56" s="3" t="n"/>
       <c r="L56" s="3" t="n"/>
       <c r="M56" s="3" t="n"/>
+      <c r="N56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
@@ -3218,24 +3139,25 @@
       <c r="F57" s="7" t="inlineStr"/>
       <c r="G57" s="7" t="inlineStr"/>
       <c r="H57" s="7" t="inlineStr"/>
-      <c r="I57" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I57" s="7" t="inlineStr"/>
       <c r="J57" s="9" t="inlineStr">
         <is>
           <t>579-MCP4921-E/P</t>
         </is>
       </c>
-      <c r="K57" s="11" t="n">
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>MCP4921-E/P-ND</t>
+        </is>
+      </c>
+      <c r="L57" s="11" t="n">
         <v>3.25</v>
       </c>
-      <c r="L57" s="11">
-        <f>E57*K57</f>
-        <v/>
-      </c>
-      <c r="M57" s="9" t="inlineStr">
+      <c r="M57" s="11">
+        <f>E57*L57</f>
+        <v/>
+      </c>
+      <c r="N57" s="9" t="inlineStr">
         <is>
           <t>1 + 1 spare</t>
         </is>
@@ -3268,24 +3190,21 @@
       <c r="F58" s="7" t="inlineStr"/>
       <c r="G58" s="7" t="inlineStr"/>
       <c r="H58" s="7" t="inlineStr"/>
-      <c r="I58" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I58" s="7" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr">
         <is>
           <t>603-MFR-25FRF52-1K5</t>
         </is>
       </c>
-      <c r="K58" s="11" t="n">
+      <c r="K58" s="9" t="inlineStr"/>
+      <c r="L58" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="L58" s="11">
-        <f>E58*K58</f>
-        <v/>
-      </c>
-      <c r="M58" s="9" t="inlineStr">
+      <c r="M58" s="11">
+        <f>E58*L58</f>
+        <v/>
+      </c>
+      <c r="N58" s="9" t="inlineStr">
         <is>
           <t>DAC output to MC1496 pin 1</t>
         </is>
@@ -3318,24 +3237,25 @@
       <c r="F59" s="7" t="inlineStr"/>
       <c r="G59" s="7" t="inlineStr"/>
       <c r="H59" s="7" t="inlineStr"/>
-      <c r="I59" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I59" s="7" t="inlineStr"/>
       <c r="J59" s="9" t="inlineStr">
         <is>
           <t>871-B32921C3684K</t>
         </is>
       </c>
-      <c r="K59" s="11" t="n">
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>495-1395-ND</t>
+        </is>
+      </c>
+      <c r="L59" s="11" t="n">
         <v>1.2</v>
       </c>
-      <c r="L59" s="11">
-        <f>E59*K59</f>
-        <v/>
-      </c>
-      <c r="M59" s="9" t="inlineStr">
+      <c r="M59" s="11">
+        <f>E59*L59</f>
+        <v/>
+      </c>
+      <c r="N59" s="9" t="inlineStr">
         <is>
           <t>DAC reconstruction LPF + 1 spare</t>
         </is>
@@ -3363,6 +3283,7 @@
       <c r="K60" s="3" t="n"/>
       <c r="L60" s="3" t="n"/>
       <c r="M60" s="3" t="n"/>
+      <c r="N60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
@@ -3391,24 +3312,25 @@
       <c r="F61" s="7" t="inlineStr"/>
       <c r="G61" s="7" t="inlineStr"/>
       <c r="H61" s="7" t="inlineStr"/>
-      <c r="I61" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I61" s="7" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr">
         <is>
           <t>80-C320C104K5R</t>
         </is>
       </c>
-      <c r="K61" s="11" t="n">
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>399-9866-ND</t>
+        </is>
+      </c>
+      <c r="L61" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="L61" s="11">
-        <f>E61*K61</f>
-        <v/>
-      </c>
-      <c r="M61" s="9" t="inlineStr">
+      <c r="M61" s="11">
+        <f>E61*L61</f>
+        <v/>
+      </c>
+      <c r="N61" s="9" t="inlineStr">
         <is>
           <t>1 at MC1496 pin 7 + 4 at LM7171 supplies + 1 at MCP4921 + spares</t>
         </is>
@@ -3441,24 +3363,25 @@
       <c r="F62" s="7" t="inlineStr"/>
       <c r="G62" s="7" t="inlineStr"/>
       <c r="H62" s="7" t="inlineStr"/>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I62" s="7" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr">
         <is>
           <t>80-T350F106K025AT</t>
         </is>
       </c>
-      <c r="K62" s="11" t="n">
+      <c r="K62" s="9" t="inlineStr">
+        <is>
+          <t>399-3801-ND</t>
+        </is>
+      </c>
+      <c r="L62" s="11" t="n">
         <v>0.85</v>
       </c>
-      <c r="L62" s="11">
-        <f>E62*K62</f>
-        <v/>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
+      <c r="M62" s="11">
+        <f>E62*L62</f>
+        <v/>
+      </c>
+      <c r="N62" s="9" t="inlineStr">
         <is>
           <t>Bulk: +12V, -8.3V, +5V, +3.3V</t>
         </is>
@@ -3486,6 +3409,7 @@
       <c r="K63" s="3" t="n"/>
       <c r="L63" s="3" t="n"/>
       <c r="M63" s="3" t="n"/>
+      <c r="N63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -3514,24 +3438,25 @@
       <c r="F64" s="7" t="inlineStr"/>
       <c r="G64" s="7" t="inlineStr"/>
       <c r="H64" s="7" t="inlineStr"/>
-      <c r="I64" s="12" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I64" s="7" t="inlineStr"/>
       <c r="J64" s="12" t="inlineStr">
         <is>
           <t>651-1715022</t>
         </is>
       </c>
-      <c r="K64" s="13" t="n">
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>277-1273-ND</t>
+        </is>
+      </c>
+      <c r="L64" s="13" t="n">
         <v>1.85</v>
       </c>
-      <c r="L64" s="13">
-        <f>E64*K64</f>
-        <v/>
-      </c>
-      <c r="M64" s="12" t="inlineStr">
+      <c r="M64" s="13">
+        <f>E64*L64</f>
+        <v/>
+      </c>
+      <c r="N64" s="12" t="inlineStr">
         <is>
           <t>+12V, +5V, -8.3V, -90V (bias), GND</t>
         </is>
@@ -3564,24 +3489,25 @@
       <c r="F65" s="7" t="inlineStr"/>
       <c r="G65" s="7" t="inlineStr"/>
       <c r="H65" s="7" t="inlineStr"/>
-      <c r="I65" s="12" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I65" s="7" t="inlineStr"/>
       <c r="J65" s="12" t="inlineStr">
         <is>
           <t>512-1N4738A</t>
         </is>
       </c>
-      <c r="K65" s="13" t="n">
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>1N4738A-TPCT-ND</t>
+        </is>
+      </c>
+      <c r="L65" s="13" t="n">
         <v>0.18</v>
       </c>
-      <c r="L65" s="13">
-        <f>E65*K65</f>
-        <v/>
-      </c>
-      <c r="M65" s="12" t="inlineStr">
+      <c r="M65" s="13">
+        <f>E65*L65</f>
+        <v/>
+      </c>
+      <c r="N65" s="12" t="inlineStr">
         <is>
           <t>-8.3V derivation from -90V + spares</t>
         </is>
@@ -3614,24 +3540,21 @@
       <c r="F66" s="7" t="inlineStr"/>
       <c r="G66" s="7" t="inlineStr"/>
       <c r="H66" s="7" t="inlineStr"/>
-      <c r="I66" s="12" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I66" s="7" t="inlineStr"/>
       <c r="J66" s="12" t="inlineStr">
         <is>
           <t>603-PR01000101502JR500</t>
         </is>
       </c>
-      <c r="K66" s="13" t="n">
+      <c r="K66" s="12" t="inlineStr"/>
+      <c r="L66" s="13" t="n">
         <v>0.55</v>
       </c>
-      <c r="L66" s="13">
-        <f>E66*K66</f>
-        <v/>
-      </c>
-      <c r="M66" s="12" t="inlineStr">
+      <c r="M66" s="13">
+        <f>E66*L66</f>
+        <v/>
+      </c>
+      <c r="N66" s="12" t="inlineStr">
         <is>
           <t>-8.3V dropper from -90V rail + 1 spare</t>
         </is>
@@ -3659,6 +3582,7 @@
       <c r="K67" s="3" t="n"/>
       <c r="L67" s="3" t="n"/>
       <c r="M67" s="3" t="n"/>
+      <c r="N67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
@@ -3687,24 +3611,25 @@
       <c r="F68" s="7" t="inlineStr"/>
       <c r="G68" s="7" t="inlineStr"/>
       <c r="H68" s="7" t="inlineStr"/>
-      <c r="I68" s="14" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I68" s="7" t="inlineStr"/>
       <c r="J68" s="14" t="inlineStr">
         <is>
           <t>649-69190-403HLF</t>
         </is>
       </c>
-      <c r="K68" s="16" t="n">
+      <c r="K68" s="14" t="inlineStr">
+        <is>
+          <t>S1011E-03-ND</t>
+        </is>
+      </c>
+      <c r="L68" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="L68" s="16">
-        <f>E68*K68</f>
-        <v/>
-      </c>
-      <c r="M68" s="14" t="inlineStr">
+      <c r="M68" s="16">
+        <f>E68*L68</f>
+        <v/>
+      </c>
+      <c r="N68" s="14" t="inlineStr">
         <is>
           <t>RF output to driver: HOT+, HOT-, GND</t>
         </is>
@@ -3737,24 +3662,25 @@
       <c r="F69" s="7" t="inlineStr"/>
       <c r="G69" s="7" t="inlineStr"/>
       <c r="H69" s="7" t="inlineStr"/>
-      <c r="I69" s="14" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I69" s="7" t="inlineStr"/>
       <c r="J69" s="14" t="inlineStr">
         <is>
           <t>649-69190-405HLF</t>
         </is>
       </c>
-      <c r="K69" s="16" t="n">
+      <c r="K69" s="14" t="inlineStr">
+        <is>
+          <t>S1011E-05-ND</t>
+        </is>
+      </c>
+      <c r="L69" s="16" t="n">
         <v>0.55</v>
       </c>
-      <c r="L69" s="16">
-        <f>E69*K69</f>
-        <v/>
-      </c>
-      <c r="M69" s="14" t="inlineStr">
+      <c r="M69" s="16">
+        <f>E69*L69</f>
+        <v/>
+      </c>
+      <c r="N69" s="14" t="inlineStr">
         <is>
           <t>SPI to MCU: SCK, MOSI, CS, LDAC, GND</t>
         </is>
@@ -3787,24 +3713,25 @@
       <c r="F70" s="7" t="inlineStr"/>
       <c r="G70" s="7" t="inlineStr"/>
       <c r="H70" s="7" t="inlineStr"/>
-      <c r="I70" s="14" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I70" s="7" t="inlineStr"/>
       <c r="J70" s="14" t="inlineStr">
         <is>
           <t>649-69190-402HLF</t>
         </is>
       </c>
-      <c r="K70" s="16" t="n">
+      <c r="K70" s="14" t="inlineStr">
+        <is>
+          <t>S1011E-02-ND</t>
+        </is>
+      </c>
+      <c r="L70" s="16" t="n">
         <v>0.45</v>
       </c>
-      <c r="L70" s="16">
-        <f>E70*K70</f>
-        <v/>
-      </c>
-      <c r="M70" s="14" t="inlineStr">
+      <c r="M70" s="16">
+        <f>E70*L70</f>
+        <v/>
+      </c>
+      <c r="N70" s="14" t="inlineStr">
         <is>
           <t>Paddle dit/dah input (or use jumper wires)</t>
         </is>
@@ -3837,24 +3764,21 @@
       <c r="F71" s="7" t="inlineStr"/>
       <c r="G71" s="7" t="inlineStr"/>
       <c r="H71" s="7" t="inlineStr"/>
-      <c r="I71" s="14" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="14" t="inlineStr">
         <is>
           <t>602-9314-4-100-WT005</t>
         </is>
       </c>
-      <c r="K71" s="16" t="n">
+      <c r="K71" s="14" t="inlineStr"/>
+      <c r="L71" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="L71" s="16">
-        <f>E71*K71</f>
-        <v/>
-      </c>
-      <c r="M71" s="14" t="inlineStr">
+      <c r="M71" s="16">
+        <f>E71*L71</f>
+        <v/>
+      </c>
+      <c r="N71" s="14" t="inlineStr">
         <is>
           <t>Inter-board + paddle wiring; OWN already?</t>
         </is>
@@ -3882,6 +3806,7 @@
       <c r="K72" s="3" t="n"/>
       <c r="L72" s="3" t="n"/>
       <c r="M72" s="3" t="n"/>
+      <c r="N72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="17" t="inlineStr">
@@ -3910,37 +3835,38 @@
       <c r="F73" s="7" t="inlineStr"/>
       <c r="G73" s="7" t="inlineStr"/>
       <c r="H73" s="7" t="inlineStr"/>
-      <c r="I73" s="17" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
+      <c r="I73" s="7" t="inlineStr"/>
       <c r="J73" s="17" t="inlineStr">
         <is>
           <t>523-31-221-RFX</t>
         </is>
       </c>
-      <c r="K73" s="19" t="n">
+      <c r="K73" s="17" t="inlineStr">
+        <is>
+          <t>ACX1230-ND</t>
+        </is>
+      </c>
+      <c r="L73" s="19" t="n">
         <v>6.5</v>
       </c>
-      <c r="L73" s="19">
-        <f>E73*K73</f>
-        <v/>
-      </c>
-      <c r="M73" s="17" t="inlineStr">
+      <c r="M73" s="19">
+        <f>E73*L73</f>
+        <v/>
+      </c>
+      <c r="N73" s="17" t="inlineStr">
         <is>
           <t>Scope tap-offs at LPF out and MC1496 out (optional)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="J75" s="20" t="inlineStr">
+      <c r="K75" s="20" t="inlineStr">
         <is>
           <t>TOTAL:</t>
         </is>
       </c>
-      <c r="L75" s="21">
-        <f>SUM(L2:L73)</f>
+      <c r="M75" s="21">
+        <f>SUM(M2:M73)</f>
         <v/>
       </c>
     </row>
@@ -3955,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -4016,189 +3942,210 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  On Hand      Mark X if you already have it in stock</t>
+          <t xml:space="preserve">  On Hand       Mark X if you already have it in stock</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ordered      Mark X when the PO goes out</t>
+          <t xml:space="preserve">  Ordered       Mark X when the PO goes out</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Received     Mark X when the parts arrive</t>
+          <t xml:space="preserve">  Received      Mark X when the parts arrive</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Supplier     Mouser / Adafruit / KitsAndParts / etc.</t>
+          <t xml:space="preserve">  Ordered From  Which supplier you actually ordered from (M / DK / A / KP)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Part Number  Supplier P/N for ordering</t>
+          <t xml:space="preserve">  Mouser P/N    Mouser catalog number</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Unit $       Estimated unit price (verify when ordering)</t>
+          <t xml:space="preserve">  Digi-Key P/N  Digi-Key catalog number (where known; some parts left blank</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ext $        Auto = Qty x Unit $</t>
+          <t xml:space="preserve">                because Yageo MFR-25 axial resistor P/Ns vary by value - search</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Notes        Substitutions, matching requirements, gotchas</t>
+          <t xml:space="preserve">                Digi-Key for "Yageo MFR-25" + value + tolerance)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Unit $        Estimated unit price (verify when ordering)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
-        <is>
-          <t>Sections:</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ext $         Auto = Qty x Unit $</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  VFO     Si5351 module + jumper hardware + pi pad + 7-pole LPF + J310 buffer</t>
+          <t xml:space="preserve">  Notes         Substitutions, matching requirements, gotchas</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  KEYER   MC1496 + bias network + PNP null injection + LM7171 post-amps + MCP4921 envelope DAC</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  POWER   Power input terminal block + bulk bypass + -8.3V derivation from -90V</t>
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>Sections:</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CONN    Off-board headers (SPI, RF out, paddle)</t>
+          <t xml:space="preserve">  VFO     Si5351 module + jumper hardware + pi pad + 7-pole LPF + J310 buffer</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  TEST    Bench bring-up extras (BNC tap-offs for scope, etc.)</t>
+          <t xml:space="preserve">  KEYER   MC1496 + bias network + PNP null injection + LM7171 post-amps + MCP4921 envelope DAC</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  POWER   Power input terminal block + bulk bypass + -8.3V derivation from -90V</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
-        <is>
-          <t>Bench bring-up notes:</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONN    Off-board headers (SPI, RF out, paddle)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Bench supplies provide +12V, -8.3V, +5V (and -90V if testing on-board zener+dropper)</t>
+          <t xml:space="preserve">  TEST    Bench bring-up extras (BNC tap-offs for scope, etc.)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - First bring-up: bypass J310 source follower with 0R jumper at Q1 footprint</t>
-        </is>
-      </c>
+      <c r="A27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Match PNP transistors T1/T2 by DMM Vbe (~5mV tolerance) for cleanest carrier null</t>
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Bench bring-up notes:</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Match RLa/RLb (3.9k) by DMM for differential balance (~1% tolerance)</t>
+          <t xml:space="preserve">  - Bench supplies provide +12V, -8.3V, +5V (and -90V if testing on-board zener+dropper)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - MC1496 R4 (51 ohm at pin 1) forms divider with R_F_D (1.5k); sets envelope DAC scale</t>
+          <t xml:space="preserve">  - First bring-up: bypass J310 source follower with 0R jumper at Q1 footprint</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Match PNP transistors T1/T2 by DMM Vbe (~5mV tolerance) for cleanest carrier null</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="inlineStr">
-        <is>
-          <t>NOT included on this list (separate orders):</t>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Match RLa/RLb (3.9k) by DMM for differential balance (~1% tolerance)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - WH2004A LCD display (separate parts list when display section is built)</t>
+          <t xml:space="preserve">  - MC1496 R4 (51 ohm at pin 1) forms divider with R_F_D (1.5k); sets envelope DAC scale</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Rotary encoder + paddle key (your choice; not blocking bench bring-up)</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - MCU board (Adafruit Metro ESP32-S3 - already owned)</t>
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>NOT included on this list (separate orders):</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - PA-side parts: bias DAC MCP4728, OPA454, cathode monitor, MCP23017 GPIO expander</t>
+          <t xml:space="preserve">  - WH2004A LCD display (separate parts list when display section is built)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Rotary encoder + paddle key (your choice; not blocking bench bring-up)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - MCU board (Adafruit Metro ESP32-S3 - already owned)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - PA-side parts: bias DAC MCP4728, OPA454, cathode monitor, MCP23017 GPIO expander</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Power supply transformers, mains hardware, chassis</t>
         </is>

</xml_diff>

<commit_message>
kicad: control-board sheets — buffer_keyer keyer body, arduino SPI labels, custom-symbol plan
- buffer_keyer.kicad_sch: place MC1496 keyer support components
  (carrier divider R11/R12, modulator port R3, emitter-degen Re,
  modulator coupling C1, VEE bypass C5, R2 Iee, bypass network),
  MCP4921 envelope DAC U4 with reconstruction cap C3, terminal
  blocks J1/J2/J3 for +5V/+12V/-90V/VEE input, hierarchical labels
  for VFO_OUT, SCK, MOSI, CS_DAC.
- arduino.kicad_sch: add SCK and MOSI hierarchical outputs for SPI
  link to MCP4921. CS_DAC still TODO.
- vfo.kicad_sch + KiCAD.kicad_sch: minor edits, sheet pin updates.
- Documentation/kicad_custom_symbols.md: new doc — pattern and plan
  for project-local xmitter:Metro_ESP32S3 symbol to replace the
  cluttered stock symbol (~30 pins → 10 pins, project-named).
- VFO_Keyer_Order.xlsx: small status updates.
- xmitter_prj/keyer.sch: minor cleanup.
</commit_message>
<xml_diff>
--- a/Documentation/VFO_Keyer_Order.xlsx
+++ b/Documentation/VFO_Keyer_Order.xlsx
@@ -3236,16 +3236,16 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>5-pos screw terminal block 5.08 mm pitch</t>
+          <t>2-pos screw terminal block 5.08 mm pitch (3 blocks = 6 positions for 5 rails)</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>THT 5pos</t>
+          <t>THT 2pos × 3</t>
         </is>
       </c>
       <c r="E52" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F52" s="10" t="n"/>
       <c r="G52" s="10" t="n">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="O52" s="15" t="inlineStr">
         <is>
-          <t>+12V, +5V, -8.3V, -90V (bias), GND | 3 × 2-pos (6 positions total; need 5 — OR swap to single 5-pos 1715061)</t>
+          <t>5-pos (1715061) was out of stock; using 3 × 2-pos for 6 total positions. Suggested rail groupings: (+12V, GND) (+5V, GND) (-8.3V, -90V). Phoenix Contact MKDSN 1,5/2-5,08.</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="L63" s="23" t="inlineStr">
         <is>

</xml_diff>